<commit_message>
Refresh live data 2026-06-01T16:59Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-05-29T14:17:09Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-01T16:59:15Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-05-29T14:17:09Z</t>
+          <t>Last refreshed: 2026-06-01T16:59:15Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.48</v>
+        <v>4.45</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-29T14:17:09Z</t>
+          <t>2026-06-01T16:59:15Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>247.1699981689453</v>
+        <v>248.5249938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.04999923706055</v>
+        <v>42.2400016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>44.4099006652832</v>
+        <v>44.47990036010742</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>569.4149780273438</v>
+        <v>571.47998046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>187.5950012207031</v>
+        <v>185.2749938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-02T15:17Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-01T16:59:15Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-02T15:16:57Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-01T16:59:15Z</t>
+          <t>Last refreshed: 2026-06-02T15:16:57Z</t>
         </is>
       </c>
     </row>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.47</v>
+        <v>0.42</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-01T16:59:15Z</t>
+          <t>2026-06-02T15:16:57Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>248.5249938964844</v>
+        <v>250.7200012207031</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.2400016784668</v>
+        <v>42.54999923706055</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>44.47990036010742</v>
+        <v>44.06499862670898</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>571.47998046875</v>
+        <v>546.02001953125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>185.2749938964844</v>
+        <v>186.1000061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-03T16:14Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-02T15:16:57Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-03T15:56:59Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-02T15:16:57Z</t>
+          <t>Last refreshed: 2026-06-03T15:56:59Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.45</v>
+        <v>4.67</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-05-21T18:10:16Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-05-21T18:10:16Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.42</v>
+        <v>0.53</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-05-21T18:10:16Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-06-03T15:56:59Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-06-03T15:56:59Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-06-03T15:56:59Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-06-03T15:56:59Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.53</v>
+        <v>6.51</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-05-21T18:10:16Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-06-03T15:56:59Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-06-03T15:56:59Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-02T15:16:57Z</t>
+          <t>2026-06-03T15:56:59Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>250.7200012207031</v>
+        <v>248.8274993896484</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.54999923706055</v>
+        <v>41.11999893188477</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>44.06499862670898</v>
+        <v>46.61999893188477</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>546.02001953125</v>
+        <v>541.9199829101562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>186.1000061035156</v>
+        <v>178.6300048828125</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-04T14:33Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-03T15:56:59Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-04T14:12:08Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-03T15:56:59Z</t>
+          <t>Last refreshed: 2026-06-04T14:12:08Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-03T15:56:59Z</t>
+          <t>2026-06-04T14:12:08Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-03T15:56:59Z</t>
+          <t>2026-06-04T14:12:08Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-03T15:56:59Z</t>
+          <t>2026-06-04T14:12:08Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-03T15:56:59Z</t>
+          <t>2026-06-04T14:12:08Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-03T15:56:59Z</t>
+          <t>2026-06-04T14:12:08Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-03T15:56:59Z</t>
+          <t>2026-06-04T14:12:08Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-03T15:56:59Z</t>
+          <t>2026-06-04T14:12:08Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>248.8274993896484</v>
+        <v>253.1150054931641</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>41.11999893188477</v>
+        <v>42.34500122070312</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>46.61999893188477</v>
+        <v>47.26499938964844</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>541.9199829101562</v>
+        <v>543.375</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>178.6300048828125</v>
+        <v>184.2700042724609</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-05T14:22Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-04T14:12:08Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-05T14:04:40Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-04T14:12:08Z</t>
+          <t>Last refreshed: 2026-06-05T14:04:40Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-04T14:12:08Z</t>
+          <t>2026-06-05T14:04:40Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-04T14:12:08Z</t>
+          <t>2026-06-05T14:04:40Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-04T14:12:08Z</t>
+          <t>2026-06-05T14:04:40Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32617,12 +32617,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-04T14:12:08Z</t>
+          <t>2026-06-05T14:04:40Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32685,7 +32685,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>283207</v>
+        <v>280467</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -32709,12 +32709,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-04T14:12:08Z</t>
+          <t>2026-06-05T14:04:40Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-04T14:12:08Z</t>
+          <t>2026-06-05T14:04:40Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-04T14:12:08Z</t>
+          <t>2026-06-05T14:04:40Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>253.1150054931641</v>
+        <v>256.8200073242188</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.34500122070312</v>
+        <v>42.41999816894531</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>47.26499938964844</v>
+        <v>46.59999847412109</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>543.375</v>
+        <v>543.6400146484375</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>184.2700042724609</v>
+        <v>182.8600006103516</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-08T15:08Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-05T14:04:40Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-08T14:54:04Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-05T14:04:40Z</t>
+          <t>Last refreshed: 2026-06-08T14:54:04Z</t>
         </is>
       </c>
     </row>
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.318</v>
+        <v>16.485</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-05T14:04:40Z</t>
+          <t>2026-06-08T14:54:04Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-05T14:04:40Z</t>
+          <t>2026-06-08T14:54:04Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-05T14:04:40Z</t>
+          <t>2026-06-08T14:54:04Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-05T14:04:40Z</t>
+          <t>2026-06-08T14:54:04Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-05T14:04:40Z</t>
+          <t>2026-06-08T14:54:04Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32731,7 +32731,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>198.116</v>
+        <v>212.366</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -32755,12 +32755,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-05T14:04:40Z</t>
+          <t>2026-06-08T14:54:04Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-05T14:04:40Z</t>
+          <t>2026-06-08T14:54:04Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>256.8200073242188</v>
+        <v>254.5200042724609</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.41999816894531</v>
+        <v>42.38000106811523</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>46.59999847412109</v>
+        <v>48.65999984741211</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>543.6400146484375</v>
+        <v>559.2150268554688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>182.8600006103516</v>
+        <v>181.6999969482422</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-09T14:13Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-08T14:54:04Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-09T13:57:48Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-08T14:54:04Z</t>
+          <t>Last refreshed: 2026-06-09T13:57:48Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-08T14:54:04Z</t>
+          <t>2026-06-09T13:57:48Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-08T14:54:04Z</t>
+          <t>2026-06-09T13:57:48Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-08T14:54:04Z</t>
+          <t>2026-06-09T13:57:48Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-08T14:54:04Z</t>
+          <t>2026-06-09T13:57:48Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-08T14:54:04Z</t>
+          <t>2026-06-09T13:57:48Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-08T14:54:04Z</t>
+          <t>2026-06-09T13:57:48Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-08T14:54:04Z</t>
+          <t>2026-06-09T13:57:48Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>254.5200042724609</v>
+        <v>251.7100067138672</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.38000106811523</v>
+        <v>43.70999908447266</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>48.65999984741211</v>
+        <v>49.03720092773438</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>559.2150268554688</v>
+        <v>575.47998046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>181.6999969482422</v>
+        <v>185.375</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-10T14:47Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-09T13:57:48Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-10T14:31:56Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-09T13:57:48Z</t>
+          <t>Last refreshed: 2026-06-10T14:31:56Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-09T13:57:48Z</t>
+          <t>2026-06-10T14:31:56Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32501,7 +32501,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>177.936</v>
+        <v>180.554</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -32525,12 +32525,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-09T13:57:48Z</t>
+          <t>2026-06-10T14:31:56Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-09T13:57:48Z</t>
+          <t>2026-06-10T14:31:56Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-09T13:57:48Z</t>
+          <t>2026-06-10T14:31:56Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-09T13:57:48Z</t>
+          <t>2026-06-10T14:31:56Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-09T13:57:48Z</t>
+          <t>2026-06-10T14:31:56Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-09T13:57:48Z</t>
+          <t>2026-06-10T14:31:56Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>251.7100067138672</v>
+        <v>256.5899963378906</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.70999908447266</v>
+        <v>42.63999938964844</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>49.03720092773438</v>
+        <v>48.85499954223633</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>575.47998046875</v>
+        <v>564.6500244140625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>185.375</v>
+        <v>180.7178039550781</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-11T15:13Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-10T14:31:56Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-11T15:00:30Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-10T14:31:56Z</t>
+          <t>Last refreshed: 2026-06-11T15:00:30Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-10T14:31:56Z</t>
+          <t>2026-06-11T15:00:30Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-10T14:31:56Z</t>
+          <t>2026-06-11T15:00:30Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-10T14:31:56Z</t>
+          <t>2026-06-11T15:00:30Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-10T14:31:56Z</t>
+          <t>2026-06-11T15:00:30Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-10T14:31:56Z</t>
+          <t>2026-06-11T15:00:30Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-10T14:31:56Z</t>
+          <t>2026-06-11T15:00:30Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-10T14:31:56Z</t>
+          <t>2026-06-11T15:00:30Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>256.5899963378906</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.63999938964844</v>
+        <v>41.9900016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>48.85499954223633</v>
+        <v>50.01499938964844</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>564.6500244140625</v>
+        <v>530.2750244140625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>180.7178039550781</v>
+        <v>175.3249969482422</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-12T14:34Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-11T15:00:30Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-12T14:18:00Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-11T15:00:30Z</t>
+          <t>Last refreshed: 2026-06-12T14:18:00Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-11T15:00:30Z</t>
+          <t>2026-06-12T14:18:00Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-11T15:00:30Z</t>
+          <t>2026-06-12T14:18:00Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-11T15:00:30Z</t>
+          <t>2026-06-12T14:18:00Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-11T15:00:30Z</t>
+          <t>2026-06-12T14:18:00Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-11T15:00:30Z</t>
+          <t>2026-06-12T14:18:00Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-11T15:00:30Z</t>
+          <t>2026-06-12T14:18:00Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-11T15:00:30Z</t>
+          <t>2026-06-12T14:18:00Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>259.5</v>
+        <v>259.7698974609375</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>41.9900016784668</v>
+        <v>44.16999816894531</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>50.01499938964844</v>
+        <v>50.88999938964844</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>530.2750244140625</v>
+        <v>558.7498779296875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>175.3249969482422</v>
+        <v>183.1999969482422</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-15T16:40Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-12T14:18:00Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-15T16:23:37Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-12T14:18:00Z</t>
+          <t>Last refreshed: 2026-06-15T16:23:37Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-12T14:18:00Z</t>
+          <t>2026-06-15T16:23:37Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-12T14:18:00Z</t>
+          <t>2026-06-15T16:23:37Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-12T14:18:00Z</t>
+          <t>2026-06-15T16:23:37Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-12T14:18:00Z</t>
+          <t>2026-06-15T16:23:37Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-12T14:18:00Z</t>
+          <t>2026-06-15T16:23:37Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-12T14:18:00Z</t>
+          <t>2026-06-15T16:23:37Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-12T14:18:00Z</t>
+          <t>2026-06-15T16:23:37Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>259.7698974609375</v>
+        <v>260.0799865722656</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.16999816894531</v>
+        <v>45.81999969482422</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>50.88999938964844</v>
+        <v>52.22000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>558.7498779296875</v>
+        <v>574.2100219726562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>183.1999969482422</v>
+        <v>196.1300048828125</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-16T16:21Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-15T16:23:37Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-16T16:08:18Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-15T16:23:37Z</t>
+          <t>Last refreshed: 2026-06-16T16:08:18Z</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-15T16:23:37Z</t>
+          <t>2026-06-16T16:08:18Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-15T16:23:37Z</t>
+          <t>2026-06-16T16:08:18Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-15T16:23:37Z</t>
+          <t>2026-06-16T16:08:18Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-15T16:23:37Z</t>
+          <t>2026-06-16T16:08:18Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-15T16:23:37Z</t>
+          <t>2026-06-16T16:08:18Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-15T16:23:37Z</t>
+          <t>2026-06-16T16:08:18Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-15T16:23:37Z</t>
+          <t>2026-06-16T16:08:18Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>260.0799865722656</v>
+        <v>261.75</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.81999969482422</v>
+        <v>45.7400016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.22000122070312</v>
+        <v>52.58499908447266</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>574.2100219726562</v>
+        <v>576.9249877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>196.1300048828125</v>
+        <v>198.6499938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-17T14:31Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-16T16:08:18Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-17T14:31:01Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-16T16:08:18Z</t>
+          <t>Last refreshed: 2026-06-17T14:31:01Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.67</v>
+        <v>4.47</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-21T18:10:16Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-21T18:10:16Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.53</v>
+        <v>0.38</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-21T18:10:16Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-16T16:08:18Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-16T16:08:18Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-16T16:08:18Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-16T16:08:18Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.51</v>
+        <v>6.52</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-21T18:10:16Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-16T16:08:18Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-16T16:08:18Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-16T16:08:18Z</t>
+          <t>2026-06-17T14:31:01Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>261.75</v>
+        <v>264.1199951171875</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.7400016784668</v>
+        <v>46.59999847412109</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.58499908447266</v>
+        <v>48.72000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>576.9249877929688</v>
+        <v>578.0499877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>198.6499938964844</v>
+        <v>206.1499938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-18T14:27Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-17T14:31:01Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-18T14:27:16Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-17T14:31:01Z</t>
+          <t>Last refreshed: 2026-06-18T14:27:16Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.47</v>
+        <v>4.43</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.38</v>
+        <v>0.29</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-17T14:31:01Z</t>
+          <t>2026-06-18T14:27:16Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>264.1199951171875</v>
+        <v>261.3699951171875</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.59999847412109</v>
+        <v>46.06999969482422</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>48.72000122070312</v>
+        <v>49.47000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>578.0499877929688</v>
+        <v>575.4299926757812</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>206.1499938964844</v>
+        <v>203.3049926757812</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-19T14:24Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-18T14:27:16Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-19T14:23:47Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-18T14:27:16Z</t>
+          <t>Last refreshed: 2026-06-19T14:23:47Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.43</v>
+        <v>4.49</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.29</v>
+        <v>0.27</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.52</v>
+        <v>6.47</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-18T14:27:16Z</t>
+          <t>2026-06-19T14:23:47Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>261.3699951171875</v>
+        <v>259.8599853515625</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.06999969482422</v>
+        <v>45.4900016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>49.47000122070312</v>
+        <v>53.65999984741211</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>575.4299926757812</v>
+        <v>579.72998046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>203.3049926757812</v>
+        <v>201.5299987792969</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-22T16:07Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-19T14:23:47Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-22T16:07:37Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-19T14:23:47Z</t>
+          <t>Last refreshed: 2026-06-22T16:07:37Z</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32346,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32438,7 +32438,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-19T14:23:47Z</t>
+          <t>2026-06-22T16:07:37Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>259.8599853515625</v>
+        <v>263.7099914550781</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.4900016784668</v>
+        <v>45.88000106811523</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.65999984741211</v>
+        <v>52.54000091552734</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>579.72998046875</v>
+        <v>577.0900268554688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>201.5299987792969</v>
+        <v>201.1000061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-23T13:57Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-22T16:07:37Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-23T13:57:10Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-22T16:07:37Z</t>
+          <t>Last refreshed: 2026-06-23T13:57:10Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.49</v>
+        <v>4.46</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-22T16:07:37Z</t>
+          <t>2026-06-23T13:57:10Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>263.7099914550781</v>
+        <v>263.1000061035156</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.88000106811523</v>
+        <v>44.97999954223633</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.54000091552734</v>
+        <v>52.38000106811523</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>577.0900268554688</v>
+        <v>581.02001953125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>201.1000061035156</v>
+        <v>198.2400054931641</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-24T13:32Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-23T13:57:10Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-24T13:32:51Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-23T13:57:10Z</t>
+          <t>Last refreshed: 2026-06-24T13:32:51Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.46</v>
+        <v>4.51</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-23T13:57:10Z</t>
+          <t>2026-06-24T13:32:51Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>263.1000061035156</v>
+        <v>264.1600036621094</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.97999954223633</v>
+        <v>45.18000030517578</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.38000106811523</v>
+        <v>52.22999954223633</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>581.02001953125</v>
+        <v>592.7999877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>198.2400054931641</v>
+        <v>197.8300018310547</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-25T13:32Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-24T13:32:51Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-25T13:31:50Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-24T13:32:51Z</t>
+          <t>Last refreshed: 2026-06-25T13:31:50Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.51</v>
+        <v>4.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-24T13:32:51Z</t>
+          <t>2026-06-25T13:31:50Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>264.1600036621094</v>
+        <v>264.8099975585938</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.18000030517578</v>
+        <v>46.07500076293945</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.22999954223633</v>
+        <v>52.60499954223633</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>592.7999877929688</v>
+        <v>609.8099975585938</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>197.8300018310547</v>
+        <v>204.0899963378906</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-26T13:26Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-25T13:31:50Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-26T13:26:04Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-25T13:31:50Z</t>
+          <t>Last refreshed: 2026-06-26T13:26:04Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.5</v>
+        <v>4.41</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.485</v>
+        <v>16.508</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.47</v>
+        <v>6.49</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32731,7 +32731,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>212.366</v>
+        <v>215.116</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -32755,12 +32755,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-25T13:31:50Z</t>
+          <t>2026-06-26T13:26:04Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>264.8099975585938</v>
+        <v>260.7699890136719</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.07500076293945</v>
+        <v>46.31999969482422</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.60499954223633</v>
+        <v>52.90000152587891</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>609.8099975585938</v>
+        <v>623.7000122070312</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.0899963378906</v>
+        <v>204.8999938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-29T14:54Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-26T13:26:04Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-29T14:54:15Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-26T13:26:04Z</t>
+          <t>Last refreshed: 2026-06-29T14:54:15Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.41</v>
+        <v>4.4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>49.8</v>
+        <v>44.8</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-26T13:26:04Z</t>
+          <t>2026-06-29T14:54:15Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>260.7699890136719</v>
+        <v>265.9349975585938</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.31999969482422</v>
+        <v>47.04000091552734</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.90000152587891</v>
+        <v>54.13000106811523</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>623.7000122070312</v>
+        <v>632.3300170898438</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.8999938964844</v>
+        <v>203.4199981689453</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-06-30T13:19Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-29T14:54:15Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-06-30T13:19:35Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-29T14:54:15Z</t>
+          <t>Last refreshed: 2026-06-30T13:19:35Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.4</v>
+        <v>4.38</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-29T14:54:15Z</t>
+          <t>2026-06-30T13:19:35Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>265.9349975585938</v>
+        <v>267.9800109863281</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>47.04000091552734</v>
+        <v>47.25</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>54.13000106811523</v>
+        <v>53.15000152587891</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>632.3300170898438</v>
+        <v>638.22998046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>203.4199981689453</v>
+        <v>202.2799987792969</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-01T13:43Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-06-30T13:19:35Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-01T13:42:50Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-06-30T13:19:35Z</t>
+          <t>Last refreshed: 2026-07-01T13:42:50Z</t>
         </is>
       </c>
     </row>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.28</v>
+        <v>0.3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-30T13:19:35Z</t>
+          <t>2026-07-01T13:42:50Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>267.9800109863281</v>
+        <v>271.2449951171875</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>47.25</v>
+        <v>45.60499954223633</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.15000152587891</v>
+        <v>52.29000091552734</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>638.22998046875</v>
+        <v>635.094970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>202.2799987792969</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-02T13:13Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-01T13:42:50Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-02T13:13:18Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-01T13:42:50Z</t>
+          <t>Last refreshed: 2026-07-02T13:13:18Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.38</v>
+        <v>4.44</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-01T13:42:50Z</t>
+          <t>2026-07-02T13:13:18Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>271.2449951171875</v>
+        <v>274.1400146484375</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.60499954223633</v>
+        <v>46.08000183105469</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.29000091552734</v>
+        <v>51.81999969482422</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>635.094970703125</v>
+        <v>655.719970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>201</v>
+        <v>204.8200073242188</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-03T13:17Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-02T13:13:18Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-03T13:17:44Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-02T13:13:18Z</t>
+          <t>Last refreshed: 2026-07-03T13:17:44Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.44</v>
+        <v>4.48</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32593,7 +32593,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -32617,12 +32617,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.49</v>
+        <v>6.43</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32685,7 +32685,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>280467</v>
+        <v>293209</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -32709,12 +32709,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-02T13:13:18Z</t>
+          <t>2026-07-03T13:17:44Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>274.1400146484375</v>
+        <v>279.4800109863281</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.08000183105469</v>
+        <v>45.31999969482422</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>51.81999969482422</v>
+        <v>50.97999954223633</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>655.719970703125</v>
+        <v>657.1199951171875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.8200073242188</v>
+        <v>205.1199951171875</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-06T14:40Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-03T13:17:44Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-06T14:39:59Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-03T13:17:44Z</t>
+          <t>Last refreshed: 2026-07-06T14:39:59Z</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32346,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32438,7 +32438,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.508</v>
+        <v>16.949</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-03T13:17:44Z</t>
+          <t>2026-07-06T14:39:59Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>279.4800109863281</v>
+        <v>278.5799865722656</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.31999969482422</v>
+        <v>45.66320037841797</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>50.97999954223633</v>
+        <v>49.7599983215332</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>657.1199951171875</v>
+        <v>658.875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>205.1199951171875</v>
+        <v>204.6999969482422</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-07T13:30Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-06T14:39:59Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-07T13:30:08Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-06T14:39:59Z</t>
+          <t>Last refreshed: 2026-07-07T13:30:08Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.48</v>
+        <v>4.49</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-06T14:39:59Z</t>
+          <t>2026-07-07T13:30:08Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>278.5799865722656</v>
+        <v>280.7049865722656</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.66320037841797</v>
+        <v>46.41500091552734</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>49.7599983215332</v>
+        <v>51.43000030517578</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>658.875</v>
+        <v>657.2000122070312</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.6999969482422</v>
+        <v>208.4799957275391</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-08T12:56Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-07T13:30:08Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-08T12:56:39Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-07T13:30:08Z</t>
+          <t>Last refreshed: 2026-07-08T12:56:39Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.49</v>
+        <v>4.48</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-07T13:30:08Z</t>
+          <t>2026-07-08T12:56:39Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>280.7049865722656</v>
+        <v>280.1099853515625</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.41500091552734</v>
+        <v>45.40000152587891</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>51.43000030517578</v>
+        <v>51.04999923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>657.2000122070312</v>
+        <v>646.5800170898438</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>208.4799957275391</v>
+        <v>202.8899993896484</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-09T14:01Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-08T12:56:39Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-09T14:01:23Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-08T12:56:39Z</t>
+          <t>Last refreshed: 2026-07-09T14:01:23Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.48</v>
+        <v>4.55</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32777,7 +32777,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7.36</v>
+        <v>7.47</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -32801,12 +32801,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-08T12:56:39Z</t>
+          <t>2026-07-09T14:01:23Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>280.1099853515625</v>
+        <v>279.5899963378906</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.40000152587891</v>
+        <v>44.81000137329102</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>51.04999923706055</v>
+        <v>50.70500183105469</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>646.5800170898438</v>
+        <v>624.030029296875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>202.8899993896484</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-10T13:22Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-09T14:01:23Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-10T13:22:20Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-09T14:01:23Z</t>
+          <t>Last refreshed: 2026-07-10T13:22:20Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.55</v>
+        <v>4.56</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.43</v>
+        <v>6.49</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-09T14:01:23Z</t>
+          <t>2026-07-10T13:22:20Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>279.5899963378906</v>
+        <v>279.2000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.81000137329102</v>
+        <v>45.11000061035156</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>50.70500183105469</v>
+        <v>51.0099983215332</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>624.030029296875</v>
+        <v>627.1099853515625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>196</v>
+        <v>200.1000061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-13T13:33Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-10T13:22:20Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-13T13:33:09Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-10T13:22:20Z</t>
+          <t>Last refreshed: 2026-07-13T13:33:09Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.56</v>
+        <v>4.54</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.38</v>
+        <v>0.35</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-10T13:22:20Z</t>
+          <t>2026-07-13T13:33:09Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>279.2000122070312</v>
+        <v>282.7200012207031</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.11000061035156</v>
+        <v>45.77500152587891</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>51.0099983215332</v>
+        <v>54.59999847412109</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>627.1099853515625</v>
+        <v>630.2100219726562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>200.1000061035156</v>
+        <v>203.8000030517578</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-14T12:43Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-13T13:33:09Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-14T12:43:45Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-13T13:33:09Z</t>
+          <t>Last refreshed: 2026-07-14T12:43:45Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.54</v>
+        <v>4.56</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-13T13:33:09Z</t>
+          <t>2026-07-14T12:43:45Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>282.7200012207031</v>
+        <v>279.8800048828125</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.77500152587891</v>
+        <v>45.11999893188477</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>54.59999847412109</v>
+        <v>54.86999893188477</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>630.2100219726562</v>
+        <v>626.1300048828125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>203.8000030517578</v>
+        <v>203.0200042724609</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-15T12:47Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-14T12:43:45Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-15T12:47:09Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-14T12:43:45Z</t>
+          <t>Last refreshed: 2026-07-15T12:47:09Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.56</v>
+        <v>4.62</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.36</v>
+        <v>0.4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32501,7 +32501,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>180.554</v>
+        <v>183.36</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -32525,12 +32525,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-14T12:43:45Z</t>
+          <t>2026-07-15T12:47:09Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.11999893188477</v>
+        <v>45.34999847412109</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
Refresh live data 2026-07-16T12:57Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-15T12:47:09Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-16T12:56:47Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-15T12:47:09Z</t>
+          <t>Last refreshed: 2026-07-16T12:56:47Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.62</v>
+        <v>4.58</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-15T12:47:09Z</t>
+          <t>2026-07-16T12:56:47Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>279.8800048828125</v>
+        <v>273.9200134277344</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.34999847412109</v>
+        <v>46.34000015258789</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>54.86999893188477</v>
+        <v>58.93999862670898</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>626.1300048828125</v>
+        <v>616.280029296875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>203.0200042724609</v>
+        <v>208.8899993896484</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-17T12:38Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-16T12:56:47Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-17T12:38:50Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-16T12:56:47Z</t>
+          <t>Last refreshed: 2026-07-17T12:38:50Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.58</v>
+        <v>4.55</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-16T12:56:47Z</t>
+          <t>2026-07-17T12:38:50Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>273.9200134277344</v>
+        <v>275.4400024414062</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.34000015258789</v>
+        <v>46.79999923706055</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.93999862670898</v>
+        <v>58.47000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>616.280029296875</v>
+        <v>637.5499877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>208.8899993896484</v>
+        <v>211.9299926757812</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-20T13:21Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-17T12:38:50Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-20T13:21:44Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-17T12:38:50Z</t>
+          <t>Last refreshed: 2026-07-20T13:21:44Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.55</v>
+        <v>4.57</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.41</v>
+        <v>0.37</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-17T12:38:50Z</t>
+          <t>2026-07-20T13:21:44Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>275.4400024414062</v>
+        <v>276.8399963378906</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>46.79999923706055</v>
+        <v>45.63999938964844</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.47000122070312</v>
+        <v>57.33000183105469</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>637.5499877929688</v>
+        <v>640</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>211.9299926757812</v>
+        <v>208.0299987792969</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-21T12:48Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-20T13:21:44Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-21T12:48:33Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-20T13:21:44Z</t>
+          <t>Last refreshed: 2026-07-21T12:48:33Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.57</v>
+        <v>4.55</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.37</v>
+        <v>0.39</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-20T13:21:44Z</t>
+          <t>2026-07-21T12:48:33Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>276.8399963378906</v>
+        <v>275.4700012207031</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.63999938964844</v>
+        <v>45.52000045776367</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>57.33000183105469</v>
+        <v>55.90999984741211</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>640</v>
+        <v>615.75</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>208.0299987792969</v>
+        <v>206.7700042724609</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-22T12:52Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-21T12:48:33Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-22T12:52:38Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-21T12:48:33Z</t>
+          <t>Last refreshed: 2026-07-22T12:52:38Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.55</v>
+        <v>4.6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32392,7 +32392,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-21T12:48:33Z</t>
+          <t>2026-07-22T12:52:38Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>275.4700012207031</v>
+        <v>275.8399963378906</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>45.52000045776367</v>
+        <v>44.43000030517578</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>55.90999984741211</v>
+        <v>57.61000061035156</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>615.75</v>
+        <v>618.47998046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>206.7700042724609</v>
+        <v>206.2200012207031</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-23T12:53Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-22T12:52:38Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-23T12:53:38Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-22T12:52:38Z</t>
+          <t>Last refreshed: 2026-07-23T12:53:38Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.6</v>
+        <v>4.63</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-22T12:52:38Z</t>
+          <t>2026-07-23T12:53:38Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>275.8399963378906</v>
+        <v>273.1499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.43000030517578</v>
+        <v>44.66999816894531</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>57.61000061035156</v>
+        <v>57.45000076293945</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>618.47998046875</v>
+        <v>606.219970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>206.2200012207031</v>
+        <v>201.3600006103516</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-24T12:51Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-23T12:53:38Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-24T12:50:57Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-23T12:53:38Z</t>
+          <t>Last refreshed: 2026-07-24T12:50:57Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.63</v>
+        <v>4.67</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32392,7 +32392,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.55</v>
+        <v>6.58</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-23T12:53:38Z</t>
+          <t>2026-07-24T12:50:57Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>273.1499938964844</v>
+        <v>273.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.66999816894531</v>
+        <v>43.97000122070312</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>57.45000076293945</v>
+        <v>58.38999938964844</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>606.219970703125</v>
+        <v>592.5700073242188</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>201.3600006103516</v>
+        <v>199.9600067138672</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-27T13:46Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-24T12:50:57Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-27T13:46:03Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-24T12:50:57Z</t>
+          <t>Last refreshed: 2026-07-27T13:46:03Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.67</v>
+        <v>4.71</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-24T12:50:57Z</t>
+          <t>2026-07-27T13:46:03Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>273.7999877929688</v>
+        <v>277.1900024414062</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.97000122070312</v>
+        <v>43.63999938964844</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.38999938964844</v>
+        <v>59.27000045776367</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>592.5700073242188</v>
+        <v>562.60498046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>199.9600067138672</v>
+        <v>208</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-28T13:07Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-27T13:46:03Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-28T13:06:56Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-27T13:46:03Z</t>
+          <t>Last refreshed: 2026-07-28T13:06:56Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.71</v>
+        <v>4.69</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-27T13:46:03Z</t>
+          <t>2026-07-28T13:06:56Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>277.1900024414062</v>
+        <v>276.8699951171875</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.63999938964844</v>
+        <v>43.68000030517578</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>59.27000045776367</v>
+        <v>58.40000152587891</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>562.60498046875</v>
+        <v>552.72998046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>208</v>
+        <v>207.0500030517578</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-29T13:11Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-28T13:06:56Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-29T13:11:17Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-28T13:06:56Z</t>
+          <t>Last refreshed: 2026-07-29T13:11:17Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.69</v>
+        <v>4.65</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-28T13:06:56Z</t>
+          <t>2026-07-29T13:11:17Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>276.8699951171875</v>
+        <v>283.0799865722656</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.68000030517578</v>
+        <v>44.11000061035156</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.40000152587891</v>
+        <v>58.88000106811523</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>552.72998046875</v>
+        <v>558.5499877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>207.0500030517578</v>
+        <v>212.4100036621094</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-30T12:59Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-29T13:11:17Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-30T12:59:07Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-29T13:11:17Z</t>
+          <t>Last refreshed: 2026-07-30T12:59:07Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.65</v>
+        <v>4.61</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32392,7 +32392,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-29T13:11:17Z</t>
+          <t>2026-07-30T12:59:07Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>283.0799865722656</v>
+        <v>281</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.11000061035156</v>
+        <v>42.95000076293945</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.88000106811523</v>
+        <v>59.11000061035156</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>558.5499877929688</v>
+        <v>556.7100219726562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>212.4100036621094</v>
+        <v>208.7100067138672</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-07-31T13:10Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-30T12:59:07Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-07-31T13:10:11Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-30T12:59:07Z</t>
+          <t>Last refreshed: 2026-07-31T13:10:11Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.61</v>
+        <v>4.67</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.949</v>
+        <v>17.037</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.58</v>
+        <v>6.66</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32731,7 +32731,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>215.116</v>
+        <v>212.975</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -32755,12 +32755,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-30T12:59:07Z</t>
+          <t>2026-07-31T13:10:11Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281</v>
+        <v>282.4599914550781</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.95000076293945</v>
+        <v>43.47999954223633</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>59.11000061035156</v>
+        <v>58.70000076293945</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>556.7100219726562</v>
+        <v>555.6699829101562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>208.7100067138672</v>
+        <v>210.1399993896484</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-03T13:56Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-07-31T13:10:11Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-03T13:56:28Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-07-31T13:10:11Z</t>
+          <t>Last refreshed: 2026-08-03T13:56:28Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.67</v>
+        <v>4.68</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.45</v>
+        <v>0.47</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44.8</v>
+        <v>49.5</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-31T13:10:11Z</t>
+          <t>2026-08-03T13:56:28Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>282.4599914550781</v>
+        <v>282.4750061035156</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.47999954223633</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.70000076293945</v>
+        <v>58.2599983215332</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>555.6699829101562</v>
+        <v>577.7550048828125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>210.1399993896484</v>
+        <v>215.7100067138672</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-04T13:12Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-03T13:56:28Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-04T13:12:42Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-03T13:56:28Z</t>
+          <t>Last refreshed: 2026-08-04T13:12:42Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.68</v>
+        <v>4.75</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-03T13:56:28Z</t>
+          <t>2026-08-04T13:12:42Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>282.4750061035156</v>
+        <v>282.3900146484375</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.5</v>
+        <v>44.06999969482422</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.2599983215332</v>
+        <v>58.43000030517578</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>577.7550048828125</v>
+        <v>572.969970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>215.7100067138672</v>
+        <v>217.6799926757812</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-05T13:07Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-04T13:12:42Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-05T13:07:39Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-04T13:12:42Z</t>
+          <t>Last refreshed: 2026-08-05T13:07:39Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.75</v>
+        <v>4.7</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.45</v>
+        <v>0.43</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-04T13:12:42Z</t>
+          <t>2026-08-05T13:07:39Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>282.3900146484375</v>
+        <v>281.3099975585938</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.06999969482422</v>
+        <v>44.9900016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.43000030517578</v>
+        <v>57.5099983215332</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>572.969970703125</v>
+        <v>587.8499755859375</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>217.6799926757812</v>
+        <v>221.9100036621094</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-06T13:07Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-05T13:07:39Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-06T13:07:12Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-05T13:07:39Z</t>
+          <t>Last refreshed: 2026-08-06T13:07:12Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.7</v>
+        <v>4.63</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32685,7 +32685,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>293209</v>
+        <v>289448</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -32709,12 +32709,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-05T13:07:39Z</t>
+          <t>2026-08-06T13:07:12Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.3099975585938</v>
+        <v>301.5700073242188</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.9900016784668</v>
+        <v>44.7400016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>57.5099983215332</v>
+        <v>56.66999816894531</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>587.8499755859375</v>
+        <v>592.52001953125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>221.9100036621094</v>
+        <v>221.6300048828125</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-07T12:03Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-06T13:07:12Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-07T12:03:41Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-06T13:07:12Z</t>
+          <t>Last refreshed: 2026-08-07T12:03:41Z</t>
         </is>
       </c>
     </row>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.66</v>
+        <v>6.69</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-06T13:07:12Z</t>
+          <t>2026-08-07T12:03:41Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>301.5700073242188</v>
+        <v>296.3999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.7400016784668</v>
+        <v>44.06000137329102</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>56.66999816894531</v>
+        <v>58.06000137329102</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>592.52001953125</v>
+        <v>581.2999877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>221.6300048828125</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-10T12:05Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-07T12:03:41Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-10T12:05:09Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-07T12:03:41Z</t>
+          <t>Last refreshed: 2026-08-10T12:05:09Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.63</v>
+        <v>4.69</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17.037</v>
+        <v>16.782</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32593,7 +32593,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -32617,12 +32617,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-07T12:03:41Z</t>
+          <t>2026-08-10T12:05:09Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>296.3999938964844</v>
+        <v>289.5499877929688</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.06000137329102</v>
+        <v>43.72000122070312</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.06000137329102</v>
+        <v>58.18000030517578</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>581.2999877929688</v>
+        <v>585.5800170898438</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>220</v>
+        <v>217.7599945068359</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-11T12:03Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-10T12:05:09Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-11T12:02:50Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-10T12:05:09Z</t>
+          <t>Last refreshed: 2026-08-11T12:02:50Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.69</v>
+        <v>4.65</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-10T12:05:09Z</t>
+          <t>2026-08-11T12:02:50Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>289.5499877929688</v>
+        <v>287.2200012207031</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.72000122070312</v>
+        <v>43.79000091552734</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.18000030517578</v>
+        <v>58.77999877929688</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>585.5800170898438</v>
+        <v>581.25</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>217.7599945068359</v>
+        <v>218.9700012207031</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-12T12:04Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-11T12:02:50Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-12T12:04:16Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-11T12:02:50Z</t>
+          <t>Last refreshed: 2026-08-12T12:04:16Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.65</v>
+        <v>4.72</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-11T12:02:50Z</t>
+          <t>2026-08-12T12:04:16Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>287.2200012207031</v>
+        <v>281.4100036621094</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.79000091552734</v>
+        <v>43.95000076293945</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.77999877929688</v>
+        <v>58.18000030517578</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>581.25</v>
+        <v>572.2100219726562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>218.9700012207031</v>
+        <v>219.1499938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-13T12:04Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-12T12:04:16Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-13T12:04:27Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-12T12:04:16Z</t>
+          <t>Last refreshed: 2026-08-13T12:04:27Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.72</v>
+        <v>4.7</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32392,7 +32392,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32501,7 +32501,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>183.36</v>
+        <v>184.661</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -32525,12 +32525,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-12T12:04:16Z</t>
+          <t>2026-08-13T12:04:27Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.4100036621094</v>
+        <v>281.1199951171875</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.95000076293945</v>
+        <v>44.25</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.18000030517578</v>
+        <v>58.70999908447266</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>572.2100219726562</v>
+        <v>577.25</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>219.1499938964844</v>
+        <v>222.4400024414062</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-14T12:03Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-13T12:04:27Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-14T12:03:14Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-13T12:04:27Z</t>
+          <t>Last refreshed: 2026-08-14T12:03:14Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.7</v>
+        <v>4.68</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.69</v>
+        <v>6.67</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-13T12:04:27Z</t>
+          <t>2026-08-14T12:03:14Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.1199951171875</v>
+        <v>280.9200134277344</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.25</v>
+        <v>44.59999847412109</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.70999908447266</v>
+        <v>60.04999923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>577.25</v>
+        <v>582.8900146484375</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>222.4400024414062</v>
+        <v>223.8300018310547</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-17T11:46Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-14T12:03:14Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-17T11:46:02Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-14T12:03:14Z</t>
+          <t>Last refreshed: 2026-08-17T11:46:02Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.68</v>
+        <v>4.63</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.48</v>
+        <v>0.51</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-14T12:03:14Z</t>
+          <t>2026-08-17T11:46:02Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>280.9200134277344</v>
+        <v>282.3800048828125</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.59999847412109</v>
+        <v>44.90999984741211</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>60.04999923706055</v>
+        <v>59.91999816894531</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>582.8900146484375</v>
+        <v>587.27001953125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>223.8300018310547</v>
+        <v>227.3399963378906</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-18T11:46Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-17T11:46:02Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-18T11:46:10Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-17T11:46:02Z</t>
+          <t>Last refreshed: 2026-08-18T11:46:10Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.63</v>
+        <v>4.68</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.51</v>
+        <v>0.53</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-17T11:46:02Z</t>
+          <t>2026-08-18T11:46:10Z</t>
         </is>
       </c>
       <c r="I15" t="n">

</xml_diff>

<commit_message>
Refresh live data 2026-08-19T11:45Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-18T11:46:10Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-19T11:45:38Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-18T11:46:10Z</t>
+          <t>Last refreshed: 2026-08-19T11:45:38Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.68</v>
+        <v>4.72</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-18T11:46:10Z</t>
+          <t>2026-08-19T11:45:38Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>282.3800048828125</v>
+        <v>280.0700073242188</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>44.90999984741211</v>
+        <v>43.63000106811523</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>59.91999816894531</v>
+        <v>57.40000152587891</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>587.27001953125</v>
+        <v>570.5399780273438</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>227.3399963378906</v>
+        <v>221.4700012207031</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-20T11:48Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-19T11:45:38Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-20T11:47:57Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-19T11:45:38Z</t>
+          <t>Last refreshed: 2026-08-20T11:47:57Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.72</v>
+        <v>4.71</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.52</v>
+        <v>0.46</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-19T11:45:38Z</t>
+          <t>2026-08-20T11:47:57Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>280.0700073242188</v>
+        <v>278.3099975585938</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.63000106811523</v>
+        <v>43.11000061035156</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>57.40000152587891</v>
+        <v>58.95000076293945</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>570.5399780273438</v>
+        <v>583.0499877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>221.4700012207031</v>
+        <v>220.7299957275391</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-21T11:48Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-20T11:47:57Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-21T11:47:55Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-20T11:47:57Z</t>
+          <t>Last refreshed: 2026-08-21T11:47:55Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.71</v>
+        <v>4.65</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.67</v>
+        <v>6.65</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-20T11:47:57Z</t>
+          <t>2026-08-21T11:47:55Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>278.3099975585938</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.11000061035156</v>
+        <v>42.29000091552734</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.95000076293945</v>
+        <v>61.04999923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>583.0499877929688</v>
+        <v>585.8800048828125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>220.7299957275391</v>
+        <v>212.4799957275391</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-24T11:49Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-21T11:47:55Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-24T11:49:06Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-21T11:47:55Z</t>
+          <t>Last refreshed: 2026-08-24T11:49:06Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.65</v>
+        <v>4.69</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-21T11:47:55Z</t>
+          <t>2026-08-24T11:49:06Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>282</v>
+        <v>284.0400085449219</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.29000091552734</v>
+        <v>42.93000030517578</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>61.04999923706055</v>
+        <v>62.13000106811523</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>585.8800048828125</v>
+        <v>601.0499877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>212.4799957275391</v>
+        <v>217.9100036621094</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-25T11:50Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-24T11:49:06Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-25T11:50:10Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-24T11:49:06Z</t>
+          <t>Last refreshed: 2026-08-25T11:50:10Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.69</v>
+        <v>4.74</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5</v>
+        <v>0.46</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-24T11:49:06Z</t>
+          <t>2026-08-25T11:50:10Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>284.0400085449219</v>
+        <v>287.8099975585938</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.93000030517578</v>
+        <v>42.45000076293945</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>62.13000106811523</v>
+        <v>62.79999923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>601.0499877929688</v>
+        <v>603.0700073242188</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>217.9100036621094</v>
+        <v>216.2700042724609</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-26T11:52Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-25T11:50:10Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-26T11:52:07Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-25T11:50:10Z</t>
+          <t>Last refreshed: 2026-08-26T11:52:07Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.74</v>
+        <v>4.7</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-25T11:50:10Z</t>
+          <t>2026-08-26T11:52:07Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>287.8099975585938</v>
+        <v>285.1499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.45000076293945</v>
+        <v>42.59999847412109</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>62.79999923706055</v>
+        <v>64.22000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>603.0700073242188</v>
+        <v>604.260009765625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>216.2700042724609</v>
+        <v>216.2400054931641</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-27T21:04Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-26T11:52:07Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-27T21:03:55Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-26T11:52:07Z</t>
+          <t>Last refreshed: 2026-08-27T21:03:55Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.7</v>
+        <v>4.66</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.782</v>
+        <v>16.757</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.65</v>
+        <v>6.66</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32731,7 +32731,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>212.975</v>
+        <v>207.457</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -32755,12 +32755,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-26T11:52:07Z</t>
+          <t>2026-08-27T21:03:55Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.1499938964844</v>
+        <v>285.4100036621094</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.59999847412109</v>
+        <v>42.7400016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>64.22000122070312</v>
+        <v>62.63999938964844</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>604.260009765625</v>
+        <v>600.47998046875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>216.2400054931641</v>
+        <v>216.6699981689453</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-28T21:27Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-27T21:03:55Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-28T21:27:20Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-27T21:03:55Z</t>
+          <t>Last refreshed: 2026-08-28T21:27:20Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.66</v>
+        <v>4.67</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.47</v>
+        <v>0.39</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>49.5</v>
+        <v>55.2</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-27T21:03:55Z</t>
+          <t>2026-08-28T21:27:20Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.4100036621094</v>
+        <v>285.6499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.7400016784668</v>
+        <v>42.18000030517578</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>62.63999938964844</v>
+        <v>62.11000061035156</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>600.47998046875</v>
+        <v>594.8900146484375</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>216.6699981689453</v>
+        <v>215.6699981689453</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-08-31T18:02Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-28T21:27:20Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-08-31T18:02:21Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-28T21:27:20Z</t>
+          <t>Last refreshed: 2026-08-31T18:02:21Z</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32346,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32438,7 +32438,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-28T21:27:20Z</t>
+          <t>2026-08-31T18:02:21Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.6499938964844</v>
+        <v>281.7749938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.18000030517578</v>
+        <v>42.10499954223633</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>62.11000061035156</v>
+        <v>61.72000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>594.8900146484375</v>
+        <v>594.6099853515625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>215.6699981689453</v>
+        <v>214.37890625</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-01T15:29Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-08-31T18:02:21Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-01T15:29:09Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-08-31T18:02:21Z</t>
+          <t>Last refreshed: 2026-09-01T15:29:09Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.67</v>
+        <v>4.73</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.39</v>
+        <v>0.41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-31T18:02:21Z</t>
+          <t>2026-09-01T15:29:09Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.7749938964844</v>
+        <v>281.5899963378906</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.10499954223633</v>
+        <v>42.08499908447266</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>61.72000122070312</v>
+        <v>60.78499984741211</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>594.6099853515625</v>
+        <v>596.8599853515625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>214.37890625</v>
+        <v>213</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-02T15:09Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-01T15:29:09Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-02T15:09:30Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-01T15:29:09Z</t>
+          <t>Last refreshed: 2026-09-02T15:09:30Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.73</v>
+        <v>4.75</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-01T15:29:09Z</t>
+          <t>2026-09-02T15:09:30Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.5899963378906</v>
+        <v>285.8200073242188</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.08499908447266</v>
+        <v>43.34000015258789</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>60.78499984741211</v>
+        <v>61.4900016784668</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>596.8599853515625</v>
+        <v>607.77001953125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>213</v>
+        <v>219.3800048828125</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-03T15:03Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-02T15:09:30Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-03T15:03:42Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-02T15:09:30Z</t>
+          <t>Last refreshed: 2026-09-03T15:03:42Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.75</v>
+        <v>4.79</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32685,7 +32685,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>289448</v>
+        <v>297771</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -32709,12 +32709,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-02T15:09:30Z</t>
+          <t>2026-09-03T15:03:42Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.8200073242188</v>
+        <v>286.8150024414062</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.34000015258789</v>
+        <v>43.25</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>61.4900016784668</v>
+        <v>61.54000091552734</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>607.77001953125</v>
+        <v>609.0700073242188</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>219.3800048828125</v>
+        <v>218.5500030517578</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-04T15:00Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-03T15:03:42Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-04T15:00:44Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-03T15:03:42Z</t>
+          <t>Last refreshed: 2026-09-04T15:00:44Z</t>
         </is>
       </c>
     </row>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4</v>
+        <v>0.43</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32617,12 +32617,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.66</v>
+        <v>6.71</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-03T15:03:42Z</t>
+          <t>2026-09-04T15:00:44Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>286.8150024414062</v>
+        <v>285.7699890136719</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.25</v>
+        <v>43.70000076293945</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>61.54000091552734</v>
+        <v>62.43999862670898</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>609.0700073242188</v>
+        <v>606.2449951171875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>218.5500030517578</v>
+        <v>219.2050018310547</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>